<commit_message>
Add underwriting sensitivity analysis tab
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XQgWoayZBeeG4UZmsDpVjR
</commit_message>
<xml_diff>
--- a/Commercial_Credit_Underwriting_Model.xlsx
+++ b/Commercial_Credit_Underwriting_Model.xlsx
@@ -15,6 +15,7 @@
     <sheet name="06 Collateral LTV" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="07 Risk Rating" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="08 Credit Memo" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="09 Sensitivity Analysis" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -135,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -245,6 +246,12 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2813,4 +2820,540 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Sensitivity / Downside Scenario Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>How does the credit hold up if performance weakens?</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Scenario Stress Drivers  (blue = inputs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Assumption</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Base Case</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Downside</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Comment</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Revenue Decline vs. 2025</t>
+        </is>
+      </c>
+      <c r="B6" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="27" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="D6" s="27" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E6" s="18" t="inlineStr">
+        <is>
+          <t>Lower repair volumes / lost customers</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>EBITDA Margin Compression (pts)</t>
+        </is>
+      </c>
+      <c r="B7" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="27" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D7" s="27" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="E7" s="18" t="inlineStr">
+        <is>
+          <t>Pricing pressure, wage/parts inflation</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Additional Operating Expenses ($)</t>
+        </is>
+      </c>
+      <c r="B8" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="23" t="n">
+        <v>20000</v>
+      </c>
+      <c r="D8" s="23" t="n">
+        <v>50000</v>
+      </c>
+      <c r="E8" s="18" t="inlineStr">
+        <is>
+          <t>Fuel, insurance, repairs above plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Shared Model Inputs  (pulled live from other tabs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>2025 Base Revenue</t>
+        </is>
+      </c>
+      <c r="B12" s="20">
+        <f>'02 Income Statement'!D5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>2025 Base EBITDA Margin</t>
+        </is>
+      </c>
+      <c r="B13" s="17">
+        <f>'02 Income Statement'!D9/'02 Income Statement'!D5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Depreciation &amp; Amortization</t>
+        </is>
+      </c>
+      <c r="B14" s="20">
+        <f>'02 Income Statement'!D10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Interest Expense</t>
+        </is>
+      </c>
+      <c r="B15" s="20">
+        <f>'02 Income Statement'!D12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Effective Tax Rate</t>
+        </is>
+      </c>
+      <c r="B16" s="27" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Maintenance Capex (unfinanced)</t>
+        </is>
+      </c>
+      <c r="B17" s="23" t="n">
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Total Annual Debt Service</t>
+        </is>
+      </c>
+      <c r="B18" s="20">
+        <f>'05 DSCR Analysis'!B12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>DSCR Covenant Minimum</t>
+        </is>
+      </c>
+      <c r="B19" s="19">
+        <f>'05 DSCR Analysis'!B25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Scenario Results  (recalculated CFADS &amp; DSCR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>Base Case</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>Downside</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Stressed Revenue</t>
+        </is>
+      </c>
+      <c r="B23" s="20">
+        <f>$B$12*(1-B6)</f>
+        <v/>
+      </c>
+      <c r="C23" s="20">
+        <f>$B$12*(1-C6)</f>
+        <v/>
+      </c>
+      <c r="D23" s="20">
+        <f>$B$12*(1-D6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Stressed EBITDA Margin</t>
+        </is>
+      </c>
+      <c r="B24" s="17">
+        <f>$B$13-B7</f>
+        <v/>
+      </c>
+      <c r="C24" s="17">
+        <f>$B$13-C7</f>
+        <v/>
+      </c>
+      <c r="D24" s="17">
+        <f>$B$13-D7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>EBITDA before extra OpEx</t>
+        </is>
+      </c>
+      <c r="B25" s="13">
+        <f>B23*B24</f>
+        <v/>
+      </c>
+      <c r="C25" s="13">
+        <f>C23*C24</f>
+        <v/>
+      </c>
+      <c r="D25" s="13">
+        <f>D23*D24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Less: Additional OpEx</t>
+        </is>
+      </c>
+      <c r="B26" s="13">
+        <f>-B8</f>
+        <v/>
+      </c>
+      <c r="C26" s="13">
+        <f>-C8</f>
+        <v/>
+      </c>
+      <c r="D26" s="13">
+        <f>-D8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Stressed EBITDA</t>
+        </is>
+      </c>
+      <c r="B27" s="12">
+        <f>B25+B26</f>
+        <v/>
+      </c>
+      <c r="C27" s="12">
+        <f>C25+C26</f>
+        <v/>
+      </c>
+      <c r="D27" s="12">
+        <f>D25+D26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Less: Cash Taxes</t>
+        </is>
+      </c>
+      <c r="B28" s="13">
+        <f>-MAX(0,$B$16*(B27-$B$14-$B$15))</f>
+        <v/>
+      </c>
+      <c r="C28" s="13">
+        <f>-MAX(0,$B$16*(C27-$B$14-$B$15))</f>
+        <v/>
+      </c>
+      <c r="D28" s="13">
+        <f>-MAX(0,$B$16*(D27-$B$14-$B$15))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Less: Maintenance Capex</t>
+        </is>
+      </c>
+      <c r="B29" s="13">
+        <f>-$B$17</f>
+        <v/>
+      </c>
+      <c r="C29" s="13">
+        <f>-$B$17</f>
+        <v/>
+      </c>
+      <c r="D29" s="13">
+        <f>-$B$17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>CFADS (stressed)</t>
+        </is>
+      </c>
+      <c r="B30" s="12">
+        <f>B27+B28+B29</f>
+        <v/>
+      </c>
+      <c r="C30" s="12">
+        <f>C27+C28+C29</f>
+        <v/>
+      </c>
+      <c r="D30" s="12">
+        <f>D27+D28+D29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Global DSCR</t>
+        </is>
+      </c>
+      <c r="B31" s="38">
+        <f>B30/$B$18</f>
+        <v/>
+      </c>
+      <c r="C31" s="38">
+        <f>C30/$B$18</f>
+        <v/>
+      </c>
+      <c r="D31" s="38">
+        <f>D30/$B$18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Pass / Fail Tests</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>Base Case</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>Downside</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="E34" s="6" t="inlineStr">
+        <is>
+          <t>Meaning</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>DSCR Covenant Test (&gt;= 1.20x)</t>
+        </is>
+      </c>
+      <c r="B35" s="39">
+        <f>IF(B31&gt;=$B$19,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="C35" s="39">
+        <f>IF(C31&gt;=$B$19,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="D35" s="39">
+        <f>IF(D31&gt;=$B$19,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="E35" s="18" t="inlineStr">
+        <is>
+          <t>Meets the loan's DSCR covenant</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Cash Coverage Test (&gt;= 1.00x)</t>
+        </is>
+      </c>
+      <c r="B36" s="39">
+        <f>IF(B31&gt;=1,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="C36" s="39">
+        <f>IF(C31&gt;=1,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="D36" s="39">
+        <f>IF(D31&gt;=1,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="E36" s="18" t="inlineStr">
+        <is>
+          <t>Cash flow still fully covers debt service</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="86" customHeight="1">
+      <c r="A38" s="10" t="inlineStr">
+        <is>
+          <t>Why this matters:  Underwriters never lend on the base case alone. Sensitivity (downside) analysis stresses the borrower's revenue and margins to find the breaking point and confirm the loan still services - or to size the cushion if it does not. Here the Base Case clears the 1.20x covenant; a moderate Downside breaches the covenant but cash flow still covers debt service (DSCR &gt; 1.0x); the severe Stress case fails both - the credit would then rely on collateral and the personal guarantee. This is exactly why the deal is 'Approve WITH conditions' (DSCR covenant, equity injection, collateral, guarantee) rather than an unconditional approval.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A21:E21"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A38:E38"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A10:E10"/>
+    <mergeCell ref="A33:E33"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>